<commit_message>
fix: fix de valor hora desatualizado
</commit_message>
<xml_diff>
--- a/relatorio_teste_sinosbyte.xlsx
+++ b/relatorio_teste_sinosbyte.xlsx
@@ -7,14 +7,15 @@
     <sheet sheetId="1" name="Consolidado" state="visible" r:id="rId4"/>
     <sheet sheetId="3" name="Lucas Moraes" state="visible" r:id="rId5"/>
     <sheet sheetId="4" name="Bianca Franzon" state="visible" r:id="rId6"/>
-    <sheet sheetId="5" name="João Teste 3" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Guilherme Fagundes" state="visible" r:id="rId7"/>
+    <sheet sheetId="6" name="Joszef Barrionuevo" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="64">
   <si>
     <t>CONSOLIDADO — SINOSBYTE</t>
   </si>
@@ -94,7 +95,10 @@
     <t>JUNIOR</t>
   </si>
   <si>
-    <t>João Teste 3</t>
+    <t>Guilherme Fagundes</t>
+  </si>
+  <si>
+    <t>Joszef Barrionuevo</t>
   </si>
   <si>
     <t>TOTAL GERAL</t>
@@ -166,6 +170,18 @@
     <t>TOTAL R$ MENSAL (estimado)</t>
   </si>
   <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>18:00</t>
+  </si>
+  <si>
+    <t>Teste 31</t>
+  </si>
+  <si>
+    <t>Teste 1</t>
+  </si>
+  <si>
     <t>07:45</t>
   </si>
   <si>
@@ -173,6 +189,24 @@
   </si>
   <si>
     <t>Teste 3</t>
+  </si>
+  <si>
+    <t>Teste 43211</t>
+  </si>
+  <si>
+    <t>Teste 51</t>
+  </si>
+  <si>
+    <t>Teste 361</t>
+  </si>
+  <si>
+    <t>Teste 21</t>
+  </si>
+  <si>
+    <t>Teste 41</t>
+  </si>
+  <si>
+    <t>Teste 221</t>
   </si>
 </sst>
 </file>
@@ -716,7 +750,7 @@
         <v>1</v>
       </c>
       <c r="H10" s="9">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="I10" s="10">
         <f>'Bianca Franzon'!G40</f>
@@ -751,10 +785,10 @@
         <v>1</v>
       </c>
       <c r="H11" s="9">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="I11" s="10">
-        <f>'João Teste 3'!G40</f>
+        <f>'Guilherme Fagundes'!G40</f>
       </c>
       <c r="J11" s="11">
         <f>H11*I11</f>
@@ -763,12 +797,47 @@
         <f>$H$4</f>
       </c>
     </row>
-    <row r="12" spans="8:10" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="H12" s="12" t="s">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J12" s="12">
-        <f>SUM(J9:J11)</f>
+      <c r="B12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="8">
+        <v>1</v>
+      </c>
+      <c r="H12" s="9">
+        <v>140</v>
+      </c>
+      <c r="I12" s="10">
+        <f>'Joszef Barrionuevo'!G40</f>
+      </c>
+      <c r="J12" s="11">
+        <f>H12*I12</f>
+      </c>
+      <c r="K12" s="7">
+        <f>$H$4</f>
+      </c>
+    </row>
+    <row r="13" spans="8:10" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="J13" s="12">
+        <f>SUM(J9:J12)</f>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1789,7 +1858,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1801,19 +1870,19 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>18</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>20</v>
@@ -1821,19 +1890,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" s="13">
         <f>Consolidado!H9</f>
       </c>
       <c r="G5" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H5" s="5" t="str">
         <f>Consolidado!$H$4&amp;"/"&amp;Consolidado!$E$4</f>
@@ -1842,28 +1911,28 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1894,22 +1963,22 @@
         <v>#NUM!</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G9" s="17">
         <f t="shared" si="1"/>
       </c>
       <c r="H9" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1922,22 +1991,22 @@
         <v>#NUM!</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G10" s="17">
         <f t="shared" si="1"/>
       </c>
       <c r="H10" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1950,22 +2019,22 @@
         <v>#NUM!</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G11" s="17">
         <f t="shared" si="1"/>
       </c>
       <c r="H11" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2456,7 +2525,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F40" s="18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G40" s="19">
         <f>SUM(G8:G38)</f>
@@ -2464,7 +2533,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F41" s="20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G41" s="21">
         <f>G40*E5</f>
@@ -2507,7 +2576,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2519,19 +2588,19 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>24</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>20</v>
@@ -2539,19 +2608,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" s="13">
         <f>Consolidado!H9</f>
       </c>
       <c r="G5" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H5" s="5" t="str">
         <f>Consolidado!$H$4&amp;"/"&amp;Consolidado!$E$4</f>
@@ -2560,28 +2629,28 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -2594,22 +2663,22 @@
         <v>#NUM!</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G8" s="17">
         <f t="shared" ref="G8:G38" si="1">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
       </c>
       <c r="H8" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -2621,14 +2690,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
+      <c r="C9" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G9" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="7" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
@@ -2639,14 +2718,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
+      <c r="C10" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G10" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H10" s="7"/>
+      <c r="H10" s="7" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
@@ -2658,22 +2747,22 @@
         <v>#NUM!</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G11" s="17">
         <f t="shared" si="1"/>
       </c>
       <c r="H11" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2686,22 +2775,22 @@
         <v>#NUM!</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G12" s="17">
         <f t="shared" si="1"/>
       </c>
       <c r="H12" s="7" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -2731,14 +2820,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
+      <c r="C14" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G14" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H14" s="7"/>
+      <c r="H14" s="7" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
@@ -2749,14 +2848,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
+      <c r="C15" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G15" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="7" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
@@ -2767,14 +2876,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
+      <c r="C16" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G16" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H16" s="7"/>
+      <c r="H16" s="7" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
@@ -2785,14 +2904,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
+      <c r="C17" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G17" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H17" s="7"/>
+      <c r="H17" s="7" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
@@ -2803,14 +2932,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
+      <c r="C18" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G18" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H18" s="7"/>
+      <c r="H18" s="7" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
@@ -2857,14 +2996,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
+      <c r="C21" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G21" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="7" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
@@ -2875,14 +3024,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
+      <c r="C22" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G22" s="17">
         <f t="shared" si="1"/>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="7" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
@@ -3174,7 +3333,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F40" s="18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G40" s="19">
         <f>SUM(G8:G38)</f>
@@ -3182,7 +3341,7 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F41" s="20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G41" s="21">
         <f>G40*E5</f>
@@ -3213,7 +3372,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1">
-        <f>"REGISTRO DE PONTO — João Teste 3 — SINOSBYTE — " &amp; Consolidado!$H$4 &amp; "/" &amp; Consolidado!$E$4</f>
+        <f>"REGISTRO DE PONTO — Guilherme Fagundes — SINOSBYTE — " &amp; Consolidado!$H$4 &amp; "/" &amp; Consolidado!$E$4</f>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3225,7 +3384,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3237,19 +3396,19 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>18</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>20</v>
@@ -3257,19 +3416,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" s="13">
         <f>Consolidado!H9</f>
       </c>
       <c r="G5" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H5" s="5" t="str">
         <f>Consolidado!$H$4&amp;"/"&amp;Consolidado!$E$4</f>
@@ -3278,28 +3437,28 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -3862,7 +4021,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F40" s="18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G40" s="19">
         <f>SUM(G8:G38)</f>
@@ -3870,7 +4029,695 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F41" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="G41" s="21">
+        <f>G40*E5</f>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H41"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1">
+        <f>"REGISTRO DE PONTO — Joszef Barrionuevo — SINOSBYTE — " &amp; Consolidado!$H$4 &amp; "/" &amp; Consolidado!$E$4</f>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="13">
+        <f>Consolidado!H9</f>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="5" t="str">
+        <f>Consolidado!$H$4&amp;"/"&amp;Consolidado!$E$4</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="15">
+        <f>IF(1&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,1),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B8" s="7" t="str">
+        <f t="shared" ref="B8:B38" si="0">IF(A8="","",CHOOSE(WEEKDAY(A8,2),"Segunda-feira","Terça-feira","Quarta-feira","Quinta-feira","Sexta-feira","Sábado","Domingo"))</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="17">
+        <f t="shared" ref="G8:G38" si="1">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
+      </c>
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="15">
+        <f>IF(2&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,2),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B9" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="15">
+        <f>IF(3&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,3),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B10" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H10" s="7"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="15">
+        <f>IF(4&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,4),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B11" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="15">
+        <f>IF(5&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,5),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B12" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="15">
+        <f>IF(6&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,6),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B13" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="15">
+        <f>IF(7&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,7),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B14" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H14" s="7"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="15">
+        <f>IF(8&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,8),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B15" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H15" s="7"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="15">
+        <f>IF(9&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,9),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B16" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="15">
+        <f>IF(10&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,10),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B17" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H17" s="7"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="15">
+        <f>IF(11&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,11),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B18" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="15">
+        <f>IF(12&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,12),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B19" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H19" s="7"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="15">
+        <f>IF(13&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,13),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B20" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H20" s="7"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="15">
+        <f>IF(14&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,14),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B21" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H21" s="7"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="15">
+        <f>IF(15&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,15),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B22" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H22" s="7"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="15">
+        <f>IF(16&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,16),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B23" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H23" s="7"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="15">
+        <f>IF(17&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,17),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B24" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H24" s="7"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="15">
+        <f>IF(18&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,18),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B25" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H25" s="7"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="15">
+        <f>IF(19&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,19),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B26" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H26" s="7"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="15">
+        <f>IF(20&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,20),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B27" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H27" s="7"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="15">
+        <f>IF(21&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,21),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B28" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H28" s="7"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="15">
+        <f>IF(22&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,22),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B29" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H29" s="7"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="15">
+        <f>IF(23&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,23),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B30" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H30" s="7"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="15">
+        <f>IF(24&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,24),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B31" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H31" s="7"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="15">
+        <f>IF(25&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,25),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B32" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H32" s="7"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="15">
+        <f>IF(26&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,26),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B33" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H33" s="7"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="15">
+        <f>IF(27&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,27),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B34" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C34" s="16"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H34" s="7"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="15">
+        <f>IF(28&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,28),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B35" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H35" s="7"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="15">
+        <f>IF(29&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,29),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B36" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H36" s="7"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="15">
+        <f>IF(30&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,30),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B37" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H37" s="7"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="15">
+        <f>IF(31&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,31),"")</f>
+        <v>NaN</v>
+      </c>
+      <c r="B38" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="17">
+        <f t="shared" si="1"/>
+      </c>
+      <c r="H38" s="7"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F40" s="18" t="s">
         <v>49</v>
+      </c>
+      <c r="G40" s="19">
+        <f>SUM(G8:G38)</f>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F41" s="20" t="s">
+        <v>50</v>
       </c>
       <c r="G41" s="21">
         <f>G40*E5</f>

</xml_diff>

<commit_message>
fix: caso horas iniciais não sejam informadas o sistema lida
</commit_message>
<xml_diff>
--- a/relatorio_teste_sinosbyte.xlsx
+++ b/relatorio_teste_sinosbyte.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="65">
   <si>
     <t>CONSOLIDADO — SINOSBYTE</t>
   </si>
@@ -170,28 +170,31 @@
     <t>TOTAL R$ MENSAL (estimado)</t>
   </si>
   <si>
+    <t>00:00</t>
+  </si>
+  <si>
+    <t>18:00</t>
+  </si>
+  <si>
+    <t>Teste 31</t>
+  </si>
+  <si>
+    <t>Teste 1</t>
+  </si>
+  <si>
+    <t>07:45</t>
+  </si>
+  <si>
+    <t>15:05</t>
+  </si>
+  <si>
+    <t>Teste 3</t>
+  </si>
+  <si>
+    <t>Teste 43211</t>
+  </si>
+  <si>
     <t>09:00</t>
-  </si>
-  <si>
-    <t>18:00</t>
-  </si>
-  <si>
-    <t>Teste 31</t>
-  </si>
-  <si>
-    <t>Teste 1</t>
-  </si>
-  <si>
-    <t>07:45</t>
-  </si>
-  <si>
-    <t>15:05</t>
-  </si>
-  <si>
-    <t>Teste 3</t>
-  </si>
-  <si>
-    <t>Teste 43211</t>
   </si>
   <si>
     <t>Teste 51</t>
@@ -1899,7 +1902,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="13">
-        <f>Consolidado!H9</f>
+        <v>130</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>35</v>
@@ -2617,7 +2620,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="13">
-        <f>Consolidado!H9</f>
+        <v>100</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>35</v>
@@ -2694,7 +2697,7 @@
         <v>51</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E9" s="16" t="s">
         <v>46</v>
@@ -2722,7 +2725,7 @@
         <v>51</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E10" s="16" t="s">
         <v>46</v>
@@ -2849,7 +2852,7 @@
         <v>#NUM!</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>45</v>
@@ -2877,7 +2880,7 @@
         <v>#NUM!</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D16" s="16" t="s">
         <v>45</v>
@@ -2892,7 +2895,7 @@
         <f t="shared" si="1"/>
       </c>
       <c r="H16" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -2920,7 +2923,7 @@
         <f t="shared" si="1"/>
       </c>
       <c r="H17" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -2933,7 +2936,7 @@
         <v>#NUM!</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>45</v>
@@ -2948,7 +2951,7 @@
         <f t="shared" si="1"/>
       </c>
       <c r="H18" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -3012,7 +3015,7 @@
         <f t="shared" si="1"/>
       </c>
       <c r="H21" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -3025,7 +3028,7 @@
         <v>#NUM!</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>45</v>
@@ -3040,7 +3043,7 @@
         <f t="shared" si="1"/>
       </c>
       <c r="H22" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -3425,7 +3428,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="13">
-        <f>Consolidado!H9</f>
+        <v>110</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>35</v>
@@ -4113,7 +4116,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="13">
-        <f>Consolidado!H9</f>
+        <v>140</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
fix: formatacao total coluna j
</commit_message>
<xml_diff>
--- a/relatorio_teste_sinosbyte.xlsx
+++ b/relatorio_teste_sinosbyte.xlsx
@@ -330,7 +330,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -348,6 +348,7 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -839,7 +840,7 @@
       <c r="H13" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="13">
         <f>SUM(J9:J12)</f>
       </c>
     </row>
@@ -1901,7 +1902,7 @@
       <c r="D5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="14">
         <v>130</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -1913,33 +1914,33 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
+      <c r="A8" s="16">
         <f>IF(1&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,1),"")</f>
         <v>NaN</v>
       </c>
@@ -1947,17 +1948,17 @@
         <f t="shared" ref="B8:B38" si="0">IF(A8="","",CHOOSE(WEEKDAY(A8,2),"Segunda-feira","Terça-feira","Quarta-feira","Quinta-feira","Sexta-feira","Sábado","Domingo"))</f>
         <v>#NUM!</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="17">
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="18">
         <f t="shared" ref="G8:G38" si="1">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
+      <c r="A9" s="16">
         <f>IF(2&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,2),"")</f>
         <v>NaN</v>
       </c>
@@ -1965,19 +1966,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H9" s="7" t="s">
@@ -1985,7 +1986,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+      <c r="A10" s="16">
         <f>IF(3&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,3),"")</f>
         <v>NaN</v>
       </c>
@@ -1993,19 +1994,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="G10" s="17">
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H10" s="7" t="s">
@@ -2013,7 +2014,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+      <c r="A11" s="16">
         <f>IF(4&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,4),"")</f>
         <v>NaN</v>
       </c>
@@ -2021,19 +2022,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H11" s="7" t="s">
@@ -2041,7 +2042,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="15">
+      <c r="A12" s="16">
         <f>IF(5&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,5),"")</f>
         <v>NaN</v>
       </c>
@@ -2049,17 +2050,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="17">
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
+      <c r="A13" s="16">
         <f>IF(6&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,6),"")</f>
         <v>NaN</v>
       </c>
@@ -2067,17 +2068,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="17">
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14" s="16">
         <f>IF(7&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,7),"")</f>
         <v>NaN</v>
       </c>
@@ -2085,17 +2086,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="17">
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
+      <c r="A15" s="16">
         <f>IF(8&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,8),"")</f>
         <v>NaN</v>
       </c>
@@ -2103,17 +2104,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17">
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
+      <c r="A16" s="16">
         <f>IF(9&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,9),"")</f>
         <v>NaN</v>
       </c>
@@ -2121,17 +2122,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="17">
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H16" s="7"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17" s="16">
         <f>IF(10&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,10),"")</f>
         <v>NaN</v>
       </c>
@@ -2139,17 +2140,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="17">
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H17" s="7"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18" s="16">
         <f>IF(11&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,11),"")</f>
         <v>NaN</v>
       </c>
@@ -2157,17 +2158,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="17">
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H18" s="7"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19" s="16">
         <f>IF(12&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,12),"")</f>
         <v>NaN</v>
       </c>
@@ -2175,17 +2176,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="17">
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H19" s="7"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
+      <c r="A20" s="16">
         <f>IF(13&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,13),"")</f>
         <v>NaN</v>
       </c>
@@ -2193,17 +2194,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17">
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H20" s="7"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="16">
         <f>IF(14&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,14),"")</f>
         <v>NaN</v>
       </c>
@@ -2211,17 +2212,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="17">
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H21" s="7"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
+      <c r="A22" s="16">
         <f>IF(15&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,15),"")</f>
         <v>NaN</v>
       </c>
@@ -2229,17 +2230,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="17">
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H22" s="7"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23" s="16">
         <f>IF(16&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,16),"")</f>
         <v>NaN</v>
       </c>
@@ -2247,17 +2248,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="17">
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H23" s="7"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="16">
         <f>IF(17&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,17),"")</f>
         <v>NaN</v>
       </c>
@@ -2265,17 +2266,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="17">
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H24" s="7"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25" s="16">
         <f>IF(18&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,18),"")</f>
         <v>NaN</v>
       </c>
@@ -2283,17 +2284,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="17">
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H25" s="7"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="15">
+      <c r="A26" s="16">
         <f>IF(19&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,19),"")</f>
         <v>NaN</v>
       </c>
@@ -2301,17 +2302,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="17">
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H26" s="7"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
+      <c r="A27" s="16">
         <f>IF(20&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,20),"")</f>
         <v>NaN</v>
       </c>
@@ -2319,17 +2320,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="17">
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H27" s="7"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="15">
+      <c r="A28" s="16">
         <f>IF(21&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,21),"")</f>
         <v>NaN</v>
       </c>
@@ -2337,17 +2338,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="17">
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
+      <c r="A29" s="16">
         <f>IF(22&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,22),"")</f>
         <v>NaN</v>
       </c>
@@ -2355,17 +2356,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="17">
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H29" s="7"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="15">
+      <c r="A30" s="16">
         <f>IF(23&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,23),"")</f>
         <v>NaN</v>
       </c>
@@ -2373,17 +2374,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="17">
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
+      <c r="A31" s="16">
         <f>IF(24&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,24),"")</f>
         <v>NaN</v>
       </c>
@@ -2391,17 +2392,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="17">
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
+      <c r="A32" s="16">
         <f>IF(25&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,25),"")</f>
         <v>NaN</v>
       </c>
@@ -2409,17 +2410,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="17">
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H32" s="7"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
+      <c r="A33" s="16">
         <f>IF(26&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,26),"")</f>
         <v>NaN</v>
       </c>
@@ -2427,17 +2428,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="17">
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34" s="16">
         <f>IF(27&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,27),"")</f>
         <v>NaN</v>
       </c>
@@ -2445,17 +2446,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="17">
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H34" s="7"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
+      <c r="A35" s="16">
         <f>IF(28&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,28),"")</f>
         <v>NaN</v>
       </c>
@@ -2463,17 +2464,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="17">
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H35" s="7"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="15">
+      <c r="A36" s="16">
         <f>IF(29&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,29),"")</f>
         <v>NaN</v>
       </c>
@@ -2481,17 +2482,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="17">
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H36" s="7"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="15">
+      <c r="A37" s="16">
         <f>IF(30&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,30),"")</f>
         <v>NaN</v>
       </c>
@@ -2499,17 +2500,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="17">
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H37" s="7"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="15">
+      <c r="A38" s="16">
         <f>IF(31&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,31),"")</f>
         <v>NaN</v>
       </c>
@@ -2517,28 +2518,28 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="17">
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H38" s="7"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F40" s="18" t="s">
+      <c r="F40" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="G40" s="19">
+      <c r="G40" s="20">
         <f>SUM(G8:G38)</f>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F41" s="20" t="s">
+      <c r="F41" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="G41" s="21">
+      <c r="G41" s="22">
         <f>G40*E5</f>
       </c>
     </row>
@@ -2619,7 +2620,7 @@
       <c r="D5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="14">
         <v>100</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -2631,33 +2632,33 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
+      <c r="A8" s="16">
         <f>IF(1&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,1),"")</f>
         <v>NaN</v>
       </c>
@@ -2665,19 +2666,19 @@
         <f t="shared" ref="B8:B38" si="0">IF(A8="","",CHOOSE(WEEKDAY(A8,2),"Segunda-feira","Terça-feira","Quarta-feira","Quinta-feira","Sexta-feira","Sábado","Domingo"))</f>
         <v>#NUM!</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="17">
+      <c r="G8" s="18">
         <f t="shared" ref="G8:G38" si="1">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
       </c>
       <c r="H8" s="7" t="s">
@@ -2685,7 +2686,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
+      <c r="A9" s="16">
         <f>IF(2&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,2),"")</f>
         <v>NaN</v>
       </c>
@@ -2693,19 +2694,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H9" s="7" t="s">
@@ -2713,7 +2714,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+      <c r="A10" s="16">
         <f>IF(3&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,3),"")</f>
         <v>NaN</v>
       </c>
@@ -2721,19 +2722,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="17">
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H10" s="7" t="s">
@@ -2741,7 +2742,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+      <c r="A11" s="16">
         <f>IF(4&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,4),"")</f>
         <v>NaN</v>
       </c>
@@ -2749,19 +2750,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="17">
+      <c r="G11" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H11" s="7" t="s">
@@ -2769,7 +2770,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="15">
+      <c r="A12" s="16">
         <f>IF(5&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,5),"")</f>
         <v>NaN</v>
       </c>
@@ -2777,19 +2778,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H12" s="7" t="s">
@@ -2797,7 +2798,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
+      <c r="A13" s="16">
         <f>IF(6&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,6),"")</f>
         <v>NaN</v>
       </c>
@@ -2805,17 +2806,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="17">
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14" s="16">
         <f>IF(7&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,7),"")</f>
         <v>NaN</v>
       </c>
@@ -2823,19 +2824,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F14" s="16" t="s">
+      <c r="F14" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="17">
+      <c r="G14" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H14" s="7" t="s">
@@ -2843,7 +2844,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
+      <c r="A15" s="16">
         <f>IF(8&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,8),"")</f>
         <v>NaN</v>
       </c>
@@ -2851,19 +2852,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H15" s="7" t="s">
@@ -2871,7 +2872,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
+      <c r="A16" s="16">
         <f>IF(9&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,9),"")</f>
         <v>NaN</v>
       </c>
@@ -2879,19 +2880,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="16" t="s">
+      <c r="D16" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="16" t="s">
+      <c r="E16" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="F16" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G16" s="17">
+      <c r="G16" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H16" s="7" t="s">
@@ -2899,7 +2900,7 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17" s="16">
         <f>IF(10&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,10),"")</f>
         <v>NaN</v>
       </c>
@@ -2907,19 +2908,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F17" s="16" t="s">
+      <c r="F17" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G17" s="17">
+      <c r="G17" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H17" s="7" t="s">
@@ -2927,7 +2928,7 @@
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18" s="16">
         <f>IF(11&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,11),"")</f>
         <v>NaN</v>
       </c>
@@ -2935,19 +2936,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D18" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="E18" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F18" s="16" t="s">
+      <c r="F18" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G18" s="17">
+      <c r="G18" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H18" s="7" t="s">
@@ -2955,7 +2956,7 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19" s="16">
         <f>IF(12&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,12),"")</f>
         <v>NaN</v>
       </c>
@@ -2963,17 +2964,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="17">
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H19" s="7"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
+      <c r="A20" s="16">
         <f>IF(13&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,13),"")</f>
         <v>NaN</v>
       </c>
@@ -2981,17 +2982,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17">
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H20" s="7"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="16">
         <f>IF(14&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,14),"")</f>
         <v>NaN</v>
       </c>
@@ -2999,19 +3000,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="16" t="s">
+      <c r="E21" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F21" s="16" t="s">
+      <c r="F21" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G21" s="17">
+      <c r="G21" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H21" s="7" t="s">
@@ -3019,7 +3020,7 @@
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
+      <c r="A22" s="16">
         <f>IF(15&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,15),"")</f>
         <v>NaN</v>
       </c>
@@ -3027,19 +3028,19 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="E22" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F22" s="16" t="s">
+      <c r="F22" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="G22" s="17">
+      <c r="G22" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H22" s="7" t="s">
@@ -3047,7 +3048,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23" s="16">
         <f>IF(16&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,16),"")</f>
         <v>NaN</v>
       </c>
@@ -3055,17 +3056,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="17">
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H23" s="7"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="16">
         <f>IF(17&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,17),"")</f>
         <v>NaN</v>
       </c>
@@ -3073,17 +3074,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="17">
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H24" s="7"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25" s="16">
         <f>IF(18&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,18),"")</f>
         <v>NaN</v>
       </c>
@@ -3091,17 +3092,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="17">
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H25" s="7"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="15">
+      <c r="A26" s="16">
         <f>IF(19&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,19),"")</f>
         <v>NaN</v>
       </c>
@@ -3109,17 +3110,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="17">
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H26" s="7"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
+      <c r="A27" s="16">
         <f>IF(20&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,20),"")</f>
         <v>NaN</v>
       </c>
@@ -3127,17 +3128,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="17">
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H27" s="7"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="15">
+      <c r="A28" s="16">
         <f>IF(21&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,21),"")</f>
         <v>NaN</v>
       </c>
@@ -3145,17 +3146,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="17">
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
+      <c r="A29" s="16">
         <f>IF(22&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,22),"")</f>
         <v>NaN</v>
       </c>
@@ -3163,17 +3164,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="17">
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H29" s="7"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="15">
+      <c r="A30" s="16">
         <f>IF(23&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,23),"")</f>
         <v>NaN</v>
       </c>
@@ -3181,17 +3182,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="17">
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
+      <c r="A31" s="16">
         <f>IF(24&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,24),"")</f>
         <v>NaN</v>
       </c>
@@ -3199,17 +3200,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="17">
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
+      <c r="A32" s="16">
         <f>IF(25&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,25),"")</f>
         <v>NaN</v>
       </c>
@@ -3217,17 +3218,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="17">
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H32" s="7"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
+      <c r="A33" s="16">
         <f>IF(26&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,26),"")</f>
         <v>NaN</v>
       </c>
@@ -3235,17 +3236,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="17">
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34" s="16">
         <f>IF(27&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,27),"")</f>
         <v>NaN</v>
       </c>
@@ -3253,17 +3254,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="17">
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H34" s="7"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
+      <c r="A35" s="16">
         <f>IF(28&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,28),"")</f>
         <v>NaN</v>
       </c>
@@ -3271,17 +3272,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="17">
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H35" s="7"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="15">
+      <c r="A36" s="16">
         <f>IF(29&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,29),"")</f>
         <v>NaN</v>
       </c>
@@ -3289,17 +3290,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="17">
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H36" s="7"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="15">
+      <c r="A37" s="16">
         <f>IF(30&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,30),"")</f>
         <v>NaN</v>
       </c>
@@ -3307,17 +3308,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="17">
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H37" s="7"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="15">
+      <c r="A38" s="16">
         <f>IF(31&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,31),"")</f>
         <v>NaN</v>
       </c>
@@ -3325,28 +3326,28 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="17">
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H38" s="7"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F40" s="18" t="s">
+      <c r="F40" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="G40" s="19">
+      <c r="G40" s="20">
         <f>SUM(G8:G38)</f>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F41" s="20" t="s">
+      <c r="F41" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="G41" s="21">
+      <c r="G41" s="22">
         <f>G40*E5</f>
       </c>
     </row>
@@ -3427,7 +3428,7 @@
       <c r="D5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="14">
         <v>110</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -3439,33 +3440,33 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
+      <c r="A8" s="16">
         <f>IF(1&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,1),"")</f>
         <v>NaN</v>
       </c>
@@ -3473,17 +3474,17 @@
         <f t="shared" ref="B8:B38" si="0">IF(A8="","",CHOOSE(WEEKDAY(A8,2),"Segunda-feira","Terça-feira","Quarta-feira","Quinta-feira","Sexta-feira","Sábado","Domingo"))</f>
         <v>#NUM!</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="17">
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="18">
         <f t="shared" ref="G8:G38" si="1">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
+      <c r="A9" s="16">
         <f>IF(2&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,2),"")</f>
         <v>NaN</v>
       </c>
@@ -3491,17 +3492,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="17">
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+      <c r="A10" s="16">
         <f>IF(3&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,3),"")</f>
         <v>NaN</v>
       </c>
@@ -3509,17 +3510,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="17">
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+      <c r="A11" s="16">
         <f>IF(4&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,4),"")</f>
         <v>NaN</v>
       </c>
@@ -3527,17 +3528,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="17">
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="15">
+      <c r="A12" s="16">
         <f>IF(5&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,5),"")</f>
         <v>NaN</v>
       </c>
@@ -3545,17 +3546,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="17">
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
+      <c r="A13" s="16">
         <f>IF(6&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,6),"")</f>
         <v>NaN</v>
       </c>
@@ -3563,17 +3564,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="17">
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14" s="16">
         <f>IF(7&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,7),"")</f>
         <v>NaN</v>
       </c>
@@ -3581,17 +3582,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="17">
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
+      <c r="A15" s="16">
         <f>IF(8&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,8),"")</f>
         <v>NaN</v>
       </c>
@@ -3599,17 +3600,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17">
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
+      <c r="A16" s="16">
         <f>IF(9&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,9),"")</f>
         <v>NaN</v>
       </c>
@@ -3617,17 +3618,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="17">
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H16" s="7"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17" s="16">
         <f>IF(10&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,10),"")</f>
         <v>NaN</v>
       </c>
@@ -3635,17 +3636,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="17">
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H17" s="7"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18" s="16">
         <f>IF(11&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,11),"")</f>
         <v>NaN</v>
       </c>
@@ -3653,17 +3654,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="17">
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H18" s="7"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19" s="16">
         <f>IF(12&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,12),"")</f>
         <v>NaN</v>
       </c>
@@ -3671,17 +3672,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="17">
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H19" s="7"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
+      <c r="A20" s="16">
         <f>IF(13&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,13),"")</f>
         <v>NaN</v>
       </c>
@@ -3689,17 +3690,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17">
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H20" s="7"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="16">
         <f>IF(14&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,14),"")</f>
         <v>NaN</v>
       </c>
@@ -3707,17 +3708,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="17">
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H21" s="7"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
+      <c r="A22" s="16">
         <f>IF(15&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,15),"")</f>
         <v>NaN</v>
       </c>
@@ -3725,17 +3726,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="17">
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H22" s="7"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23" s="16">
         <f>IF(16&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,16),"")</f>
         <v>NaN</v>
       </c>
@@ -3743,17 +3744,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="17">
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H23" s="7"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="16">
         <f>IF(17&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,17),"")</f>
         <v>NaN</v>
       </c>
@@ -3761,17 +3762,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="17">
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H24" s="7"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25" s="16">
         <f>IF(18&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,18),"")</f>
         <v>NaN</v>
       </c>
@@ -3779,17 +3780,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="17">
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H25" s="7"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="15">
+      <c r="A26" s="16">
         <f>IF(19&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,19),"")</f>
         <v>NaN</v>
       </c>
@@ -3797,17 +3798,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="17">
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H26" s="7"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
+      <c r="A27" s="16">
         <f>IF(20&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,20),"")</f>
         <v>NaN</v>
       </c>
@@ -3815,17 +3816,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="17">
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H27" s="7"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="15">
+      <c r="A28" s="16">
         <f>IF(21&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,21),"")</f>
         <v>NaN</v>
       </c>
@@ -3833,17 +3834,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="17">
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
+      <c r="A29" s="16">
         <f>IF(22&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,22),"")</f>
         <v>NaN</v>
       </c>
@@ -3851,17 +3852,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="17">
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H29" s="7"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="15">
+      <c r="A30" s="16">
         <f>IF(23&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,23),"")</f>
         <v>NaN</v>
       </c>
@@ -3869,17 +3870,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="17">
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
+      <c r="A31" s="16">
         <f>IF(24&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,24),"")</f>
         <v>NaN</v>
       </c>
@@ -3887,17 +3888,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="17">
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
+      <c r="A32" s="16">
         <f>IF(25&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,25),"")</f>
         <v>NaN</v>
       </c>
@@ -3905,17 +3906,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="17">
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H32" s="7"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
+      <c r="A33" s="16">
         <f>IF(26&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,26),"")</f>
         <v>NaN</v>
       </c>
@@ -3923,17 +3924,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="17">
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34" s="16">
         <f>IF(27&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,27),"")</f>
         <v>NaN</v>
       </c>
@@ -3941,17 +3942,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="17">
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H34" s="7"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
+      <c r="A35" s="16">
         <f>IF(28&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,28),"")</f>
         <v>NaN</v>
       </c>
@@ -3959,17 +3960,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="17">
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H35" s="7"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="15">
+      <c r="A36" s="16">
         <f>IF(29&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,29),"")</f>
         <v>NaN</v>
       </c>
@@ -3977,17 +3978,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="17">
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H36" s="7"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="15">
+      <c r="A37" s="16">
         <f>IF(30&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,30),"")</f>
         <v>NaN</v>
       </c>
@@ -3995,17 +3996,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="17">
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H37" s="7"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="15">
+      <c r="A38" s="16">
         <f>IF(31&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,31),"")</f>
         <v>NaN</v>
       </c>
@@ -4013,28 +4014,28 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="17">
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H38" s="7"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F40" s="18" t="s">
+      <c r="F40" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="G40" s="19">
+      <c r="G40" s="20">
         <f>SUM(G8:G38)</f>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F41" s="20" t="s">
+      <c r="F41" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="G41" s="21">
+      <c r="G41" s="22">
         <f>G40*E5</f>
       </c>
     </row>
@@ -4115,7 +4116,7 @@
       <c r="D5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="14">
         <v>140</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -4127,33 +4128,33 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
+      <c r="A8" s="16">
         <f>IF(1&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,1),"")</f>
         <v>NaN</v>
       </c>
@@ -4161,17 +4162,17 @@
         <f t="shared" ref="B8:B38" si="0">IF(A8="","",CHOOSE(WEEKDAY(A8,2),"Segunda-feira","Terça-feira","Quarta-feira","Quinta-feira","Sexta-feira","Sábado","Domingo"))</f>
         <v>#NUM!</v>
       </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="17">
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="18">
         <f t="shared" ref="G8:G38" si="1">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
       </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
+      <c r="A9" s="16">
         <f>IF(2&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,2),"")</f>
         <v>NaN</v>
       </c>
@@ -4179,17 +4180,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="17">
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
+      <c r="A10" s="16">
         <f>IF(3&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,3),"")</f>
         <v>NaN</v>
       </c>
@@ -4197,17 +4198,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="17">
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
+      <c r="A11" s="16">
         <f>IF(4&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,4),"")</f>
         <v>NaN</v>
       </c>
@@ -4215,17 +4216,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="17">
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H11" s="7"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="15">
+      <c r="A12" s="16">
         <f>IF(5&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,5),"")</f>
         <v>NaN</v>
       </c>
@@ -4233,17 +4234,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="17">
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
+      <c r="A13" s="16">
         <f>IF(6&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,6),"")</f>
         <v>NaN</v>
       </c>
@@ -4251,17 +4252,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="17">
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H13" s="7"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14" s="16">
         <f>IF(7&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,7),"")</f>
         <v>NaN</v>
       </c>
@@ -4269,17 +4270,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="17">
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
+      <c r="A15" s="16">
         <f>IF(8&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,8),"")</f>
         <v>NaN</v>
       </c>
@@ -4287,17 +4288,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="17">
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H15" s="7"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
+      <c r="A16" s="16">
         <f>IF(9&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,9),"")</f>
         <v>NaN</v>
       </c>
@@ -4305,17 +4306,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="17">
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H16" s="7"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
+      <c r="A17" s="16">
         <f>IF(10&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,10),"")</f>
         <v>NaN</v>
       </c>
@@ -4323,17 +4324,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="17">
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H17" s="7"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
+      <c r="A18" s="16">
         <f>IF(11&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,11),"")</f>
         <v>NaN</v>
       </c>
@@ -4341,17 +4342,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="17">
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H18" s="7"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
+      <c r="A19" s="16">
         <f>IF(12&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,12),"")</f>
         <v>NaN</v>
       </c>
@@ -4359,17 +4360,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="17">
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H19" s="7"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
+      <c r="A20" s="16">
         <f>IF(13&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,13),"")</f>
         <v>NaN</v>
       </c>
@@ -4377,17 +4378,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="17">
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H20" s="7"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
+      <c r="A21" s="16">
         <f>IF(14&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,14),"")</f>
         <v>NaN</v>
       </c>
@@ -4395,17 +4396,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="17">
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H21" s="7"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
+      <c r="A22" s="16">
         <f>IF(15&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,15),"")</f>
         <v>NaN</v>
       </c>
@@ -4413,17 +4414,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="17">
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H22" s="7"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
+      <c r="A23" s="16">
         <f>IF(16&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,16),"")</f>
         <v>NaN</v>
       </c>
@@ -4431,17 +4432,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="17">
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H23" s="7"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="16">
         <f>IF(17&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,17),"")</f>
         <v>NaN</v>
       </c>
@@ -4449,17 +4450,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="17">
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H24" s="7"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
+      <c r="A25" s="16">
         <f>IF(18&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,18),"")</f>
         <v>NaN</v>
       </c>
@@ -4467,17 +4468,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="17">
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H25" s="7"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="15">
+      <c r="A26" s="16">
         <f>IF(19&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,19),"")</f>
         <v>NaN</v>
       </c>
@@ -4485,17 +4486,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="17">
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H26" s="7"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
+      <c r="A27" s="16">
         <f>IF(20&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,20),"")</f>
         <v>NaN</v>
       </c>
@@ -4503,17 +4504,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="17">
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H27" s="7"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="15">
+      <c r="A28" s="16">
         <f>IF(21&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,21),"")</f>
         <v>NaN</v>
       </c>
@@ -4521,17 +4522,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="17">
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H28" s="7"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
+      <c r="A29" s="16">
         <f>IF(22&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,22),"")</f>
         <v>NaN</v>
       </c>
@@ -4539,17 +4540,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="17">
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H29" s="7"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="15">
+      <c r="A30" s="16">
         <f>IF(23&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,23),"")</f>
         <v>NaN</v>
       </c>
@@ -4557,17 +4558,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="17">
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
+      <c r="A31" s="16">
         <f>IF(24&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,24),"")</f>
         <v>NaN</v>
       </c>
@@ -4575,17 +4576,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="17">
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
+      <c r="A32" s="16">
         <f>IF(25&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,25),"")</f>
         <v>NaN</v>
       </c>
@@ -4593,17 +4594,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="17">
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H32" s="7"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
+      <c r="A33" s="16">
         <f>IF(26&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,26),"")</f>
         <v>NaN</v>
       </c>
@@ -4611,17 +4612,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="17">
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34" s="16">
         <f>IF(27&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,27),"")</f>
         <v>NaN</v>
       </c>
@@ -4629,17 +4630,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="17">
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H34" s="7"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
+      <c r="A35" s="16">
         <f>IF(28&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,28),"")</f>
         <v>NaN</v>
       </c>
@@ -4647,17 +4648,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="17">
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H35" s="7"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="15">
+      <c r="A36" s="16">
         <f>IF(29&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,29),"")</f>
         <v>NaN</v>
       </c>
@@ -4665,17 +4666,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="17">
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H36" s="7"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="15">
+      <c r="A37" s="16">
         <f>IF(30&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,30),"")</f>
         <v>NaN</v>
       </c>
@@ -4683,17 +4684,17 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="17">
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H37" s="7"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="15">
+      <c r="A38" s="16">
         <f>IF(31&lt;=DAY(EOMONTH(DATE(Consolidado!$E$4,Consolidado!$B$4,1),0)),DATE(Consolidado!$E$4,Consolidado!$B$4,31),"")</f>
         <v>NaN</v>
       </c>
@@ -4701,28 +4702,28 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="17">
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="18">
         <f t="shared" si="1"/>
       </c>
       <c r="H38" s="7"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F40" s="18" t="s">
+      <c r="F40" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="G40" s="19">
+      <c r="G40" s="20">
         <f>SUM(G8:G38)</f>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F41" s="20" t="s">
+      <c r="F41" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="G41" s="21">
+      <c r="G41" s="22">
         <f>G40*E5</f>
       </c>
     </row>

</xml_diff>

<commit_message>
entradas de teste para joszef e para guilherme
</commit_message>
<xml_diff>
--- a/relatorio_teste_sinosbyte.xlsx
+++ b/relatorio_teste_sinosbyte.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="71">
   <si>
     <t>CONSOLIDADO — SINOSBYTE</t>
   </si>
@@ -210,6 +210,24 @@
   </si>
   <si>
     <t>Teste 221</t>
+  </si>
+  <si>
+    <t>08:45</t>
+  </si>
+  <si>
+    <t>19:00</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>18:10</t>
+  </si>
+  <si>
+    <t>17:40</t>
+  </si>
+  <si>
+    <t>18:35</t>
   </si>
 </sst>
 </file>
@@ -3474,14 +3492,24 @@
         <f t="shared" ref="B8:B38" si="0">IF(A8="","",CHOOSE(WEEKDAY(A8,2),"Segunda-feira","Terça-feira","Quarta-feira","Quinta-feira","Sexta-feira","Sábado","Domingo"))</f>
         <v>#NUM!</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
+      <c r="C8" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>66</v>
+      </c>
       <c r="G8" s="18">
         <f t="shared" ref="G8:G38" si="1">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
@@ -3528,14 +3556,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
+      <c r="C11" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G11" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H11" s="7"/>
+      <c r="H11" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="16">
@@ -3546,14 +3584,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
+      <c r="C12" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>69</v>
+      </c>
       <c r="G12" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="16">
@@ -3564,14 +3612,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
+      <c r="C13" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G13" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="16">
@@ -3582,14 +3640,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
+      <c r="C14" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>66</v>
+      </c>
       <c r="G14" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H14" s="7"/>
+      <c r="H14" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="16">
@@ -3600,14 +3668,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
+      <c r="C15" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>66</v>
+      </c>
       <c r="G15" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="16">
@@ -3654,14 +3732,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
+      <c r="C18" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G18" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H18" s="7"/>
+      <c r="H18" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="16">
@@ -3672,14 +3760,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
+      <c r="C19" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>66</v>
+      </c>
       <c r="G19" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H19" s="7"/>
+      <c r="H19" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="16">
@@ -3690,14 +3788,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
+      <c r="C20" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>69</v>
+      </c>
       <c r="G20" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="16">
@@ -3708,14 +3816,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
+      <c r="C21" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G21" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="16">
@@ -3726,14 +3844,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
+      <c r="C22" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G22" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="16">
@@ -4162,14 +4290,24 @@
         <f t="shared" ref="B8:B38" si="0">IF(A8="","",CHOOSE(WEEKDAY(A8,2),"Segunda-feira","Terça-feira","Quarta-feira","Quinta-feira","Sexta-feira","Sábado","Domingo"))</f>
         <v>#NUM!</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
+      <c r="C8" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>70</v>
+      </c>
       <c r="G8" s="18">
         <f t="shared" ref="G8:G38" si="1">IF(OR(C8="",D8="",E8="",F8=""),"",(D8-C8)*24+(F8-E8)*24)</f>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
@@ -4198,14 +4336,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
+      <c r="C10" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G10" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H10" s="7"/>
+      <c r="H10" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="16">
@@ -4216,14 +4364,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
+      <c r="C11" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>70</v>
+      </c>
       <c r="G11" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H11" s="7"/>
+      <c r="H11" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="16">
@@ -4234,14 +4392,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
+      <c r="C12" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>70</v>
+      </c>
       <c r="G12" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="16">
@@ -4252,14 +4420,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
+      <c r="C13" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G13" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="16">
@@ -4270,14 +4448,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
+      <c r="C14" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>70</v>
+      </c>
       <c r="G14" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H14" s="7"/>
+      <c r="H14" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="16">
@@ -4288,14 +4476,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
+      <c r="C15" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G15" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="16">
@@ -4360,14 +4558,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
+      <c r="C19" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>70</v>
+      </c>
       <c r="G19" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H19" s="7"/>
+      <c r="H19" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="16">
@@ -4378,14 +4586,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
+      <c r="C20" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G20" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="16">
@@ -4396,14 +4614,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
+      <c r="C21" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>70</v>
+      </c>
       <c r="G21" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="16">
@@ -4414,14 +4642,24 @@
         <f t="shared" si="0"/>
         <v>#NUM!</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
+      <c r="C22" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G22" s="18">
         <f t="shared" si="1"/>
       </c>
-      <c r="H22" s="7"/>
+      <c r="H22" s="7" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="16">

</xml_diff>